<commit_message>
release: prepare version 1.03 with latest improvements
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -56,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AS13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -703,6 +706,1254 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fewygfyu3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Controlador HVAC Premium</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>45903.34375</v>
+      </c>
+      <c r="S2" t="n">
+        <v>75</v>
+      </c>
+      <c r="U2" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fwe24gvfd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sistema Batería Industrial</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>45903.3125</v>
+      </c>
+      <c r="S3" t="n">
+        <v>195</v>
+      </c>
+      <c r="U3" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fdgffdwwd3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Switch Inteligente IoT</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>100</v>
+      </c>
+      <c r="M4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>45903.25</v>
+      </c>
+      <c r="S4" t="n">
+        <v>345</v>
+      </c>
+      <c r="U4" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>JCI240001A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Termostato Digital Pro</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>45903.375</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>JCI240002B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sensor de Temperatura</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>50</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>45903.30208333334</v>
+      </c>
+      <c r="S6" t="n">
+        <v>135</v>
+      </c>
+      <c r="U6" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>JCI240003C</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Válvula Reguladora</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>100</v>
+      </c>
+      <c r="M7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>45903.20833333334</v>
+      </c>
+      <c r="S7" t="n">
+        <v>570</v>
+      </c>
+      <c r="U7" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>JCI240004D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Actuador Eléctrico</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>45903.27083333334</v>
+      </c>
+      <c r="S8" t="n">
+        <v>375</v>
+      </c>
+      <c r="U8" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>JCI240005E</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Panel de Control</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>45903.41666666666</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>JCI240006F</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Motor de Ventilación</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>45903.36458333334</v>
+      </c>
+      <c r="S10" t="n">
+        <v>90</v>
+      </c>
+      <c r="U10" t="n">
+        <v>93.8</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>JCI240007G</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Filtro de Aire Inteligente</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="M11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>45903.29166666666</v>
+      </c>
+      <c r="S11" t="n">
+        <v>240</v>
+      </c>
+      <c r="U11" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>JCI240008H</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Unidad de Control Maestra</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>45903.45833333334</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>JCI240009I</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sensor de Humedad</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>50</v>
+      </c>
+      <c r="M13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>45903.33333333334</v>
+      </c>
+      <c r="S13" t="n">
+        <v>150</v>
+      </c>
+      <c r="U13" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update: UI improvements with new features and bug fixes
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -712,90 +712,159 @@
           <t>fewygfyu3</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HVAC-CTL-TEST-001</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Controlador HVAC Premium</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Controles HVAC</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>WO-TEST-0001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BTH-TEST001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SNTEST001</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TEST-MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-HVAC-TEST-A</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>45903.34375</v>
+        <v>45903.96087520188</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>45903.96087520188</v>
+      </c>
+      <c r="R2" t="n">
+        <v>300</v>
       </c>
       <c r="S2" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>95.2</v>
+        <v>100</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X2" t="n">
         <v>0</v>
       </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF2" t="n">
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ2" t="n">
         <v>0</v>
       </c>
       <c r="AK2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
       <c r="AO2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -807,99 +876,168 @@
         <v>0</v>
       </c>
       <c r="AS2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fwe24gvfd</t>
+          <t>JCI240001A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC-CTL-2024-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sistema Batería Industrial</t>
+          <t>Controlador HVAC Inteligente</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Controles HVAC</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WO-2024-0156</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BTH-240001</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SN240001001</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FORD-MX</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Rev-C</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-HVAC-2024-A</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>66.7</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>45903.3125</v>
+        <v>45903.96087520155</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>45903.96087520156</v>
+      </c>
+      <c r="R3" t="n">
+        <v>420</v>
       </c>
       <c r="S3" t="n">
-        <v>195</v>
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>98.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X3" t="n">
         <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF3" t="n">
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ3" t="n">
         <v>0</v>
       </c>
       <c r="AK3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN3" t="n">
         <v>0</v>
       </c>
       <c r="AO3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -911,99 +1049,168 @@
         <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fdgffdwwd3</t>
+          <t>JCI240002B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BATT-SYS-2024-002</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Switch Inteligente IoT</t>
+          <t>Sistema de Gestión de Batería</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sistemas de Energía</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WO-2024-0157</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BTH-240002</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SN240002001</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>GM-MX</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Rev-B</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-BATT-2024-B</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Completado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>45903.25</v>
+        <v>45903.96087520177</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>45903.96087520178</v>
+      </c>
+      <c r="R4" t="n">
+        <v>380</v>
       </c>
       <c r="S4" t="n">
-        <v>345</v>
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>97.8</v>
+        <v>100</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB4" t="n">
         <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF4" t="n">
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
       <c r="AK4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -1015,99 +1222,168 @@
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JCI240001A</t>
+          <t>fwe24gvfd</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BATT-SYS-TEST-002</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Termostato Digital Pro</t>
+          <t>Sistema Batería Industrial</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sistemas de Energía</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>WO-TEST-0002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BTH-TEST002</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SNTEST002</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TEST-MX</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-BATT-TEST-A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
         <v>1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>45903.375</v>
+        <v>45903.960875202</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>45903.960875202</v>
+      </c>
+      <c r="R5" t="n">
+        <v>280</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
       </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB5" t="n">
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF5" t="n">
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ5" t="n">
         <v>0</v>
       </c>
       <c r="AK5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN5" t="n">
         <v>0</v>
       </c>
       <c r="AO5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
@@ -1119,99 +1395,168 @@
         <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JCI240002B</t>
+          <t>fdgffdwwd3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IOT-SWT-TEST-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sensor de Temperatura</t>
+          <t>Switch Inteligente IoT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Dispositivos IoT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>WO-TEST-0003</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BTH-TEST003</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SNTEST003</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TEST-MX</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-IOT-TEST-A</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>45903.30208333334</v>
+        <v>45903.96087520209</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>45903.96087520209</v>
+      </c>
+      <c r="R6" t="n">
+        <v>250</v>
       </c>
       <c r="S6" t="n">
-        <v>135</v>
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB6" t="n">
         <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF6" t="n">
         <v>0</v>
       </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ6" t="n">
         <v>0</v>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN6" t="n">
         <v>0</v>
       </c>
       <c r="AO6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
@@ -1223,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="AS6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -1232,90 +1577,159 @@
           <t>JCI240003C</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INT-SWT-2024-003</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Válvula Reguladora</t>
+          <t>Switch Inteligente Interior</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Controles Interiores</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WO-2024-0158</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BTH-240003</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SN240003001</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>STEL-MX</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-INT-2024-C</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Completado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>45903.20833333334</v>
+        <v>45903.96087520219</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>45903.9608752022</v>
+      </c>
+      <c r="R7" t="n">
+        <v>300</v>
       </c>
       <c r="S7" t="n">
-        <v>570</v>
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>96.3</v>
+        <v>100</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB7" t="n">
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF7" t="n">
         <v>0</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
       <c r="AK7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN7" t="n">
         <v>0</v>
       </c>
       <c r="AO7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
@@ -1327,99 +1741,168 @@
         <v>0</v>
       </c>
       <c r="AS7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JCI240004D</t>
+          <t>ther4mosta7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>THERM-ADV-2024-004</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Actuador Eléctrico</t>
+          <t>Termostato Avanzado Digital</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Controles de Temperatura</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>WO-2024-0159</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BTH-240004</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SN240004001</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NISSAN-MX</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Rev-B</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-THERM-2024-B</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>45903.27083333334</v>
+        <v>45903.96087520227</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>45903.96087520227</v>
+      </c>
+      <c r="R8" t="n">
+        <v>350</v>
       </c>
       <c r="S8" t="n">
-        <v>375</v>
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>97.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X8" t="n">
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB8" t="n">
         <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ8" t="n">
         <v>0</v>
       </c>
       <c r="AK8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN8" t="n">
         <v>0</v>
       </c>
       <c r="AO8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
@@ -1431,18 +1914,58 @@
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JCI240005E</t>
+          <t>sens0r9air2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AIR-SENS-2024-005</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Panel de Control</t>
+          <t>Sensor Calidad de Aire CO2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sensores Ambientales</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WO-2024-0160</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BTH-240005</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SN240005001</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VW-MX</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Rev-C</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-AIR-2024-C</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1457,73 +1980,102 @@
         <v>1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>45903.41666666666</v>
+        <v>45903.96087520237</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>45903.96087520239</v>
+      </c>
+      <c r="R9" t="n">
+        <v>220</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB9" t="n">
         <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF9" t="n">
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ9" t="n">
         <v>0</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN9" t="n">
         <v>0</v>
       </c>
       <c r="AO9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
@@ -1535,99 +2087,168 @@
         <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JCI240006F</t>
+          <t>act8uator5v</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ACT-HVAC-2024-006</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Motor de Ventilación</t>
+          <t>Actuador HVAC Eléctrico</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Actuadores</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>WO-2024-0161</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BTH-240006</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SN240006001</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>BMW-MX</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-ACT-2024-A</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>45903.36458333334</v>
+        <v>45903.96087520247</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>45903.96087520247</v>
+      </c>
+      <c r="R10" t="n">
+        <v>290</v>
       </c>
       <c r="S10" t="n">
-        <v>90</v>
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>93.8</v>
+        <v>100</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X10" t="n">
         <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB10" t="n">
         <v>0</v>
       </c>
       <c r="AC10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF10" t="n">
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
       <c r="AK10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN10" t="n">
         <v>0</v>
       </c>
       <c r="AO10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -1639,99 +2260,168 @@
         <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JCI240007G</t>
+          <t>disp1ay4led</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DISP-LED-2024-007</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Filtro de Aire Inteligente</t>
+          <t>Display LED Multifunción</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Interfaces Usuario</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>WO-2024-0162</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BTH-240007</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SN240007001</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TESLA-MX</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Rev-D</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-DISP-2024-D</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>66.7</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>45903.29166666666</v>
+        <v>45903.96087520256</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>45903.96087520257</v>
+      </c>
+      <c r="R11" t="n">
+        <v>410</v>
       </c>
       <c r="S11" t="n">
-        <v>240</v>
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>95.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB11" t="n">
         <v>0</v>
       </c>
       <c r="AC11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF11" t="n">
         <v>0</v>
       </c>
       <c r="AG11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ11" t="n">
         <v>0</v>
       </c>
       <c r="AK11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN11" t="n">
         <v>0</v>
       </c>
       <c r="AO11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
@@ -1743,18 +2433,58 @@
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JCI240008H</t>
+          <t>valve6flow3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VALVE-FLOW-2024-008</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unidad de Control Maestra</t>
+          <t>Válvula Control de Flujo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Válvulas de Control</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>WO-2024-0163</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>BTH-240008</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SN240008001</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>AUDI-MX</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Rev-B</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-VALVE-2024-B</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1769,73 +2499,102 @@
         <v>1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>45903.45833333334</v>
+        <v>45903.96087520264</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>45903.96087520264</v>
+      </c>
+      <c r="R12" t="n">
+        <v>365</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X12" t="n">
         <v>0</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ12" t="n">
         <v>0</v>
       </c>
       <c r="AK12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN12" t="n">
         <v>0</v>
       </c>
       <c r="AO12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
@@ -1847,99 +2606,168 @@
         <v>0</v>
       </c>
       <c r="AS12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JCI240009I</t>
+          <t>relay8power1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RELAY-PWR-2024-009</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sensor de Humedad</t>
+          <t>Relay de Potencia Industrial</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Componentes Eléctricos</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>WO-2024-0164</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>BTH-240009</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SN240009001</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MERC-MX</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Rev-A</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>JCI-SPEC-RELAY-2024-A</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>45903.33333333334</v>
+        <v>45903.96087520272</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>45903.96087520272</v>
+      </c>
+      <c r="R13" t="n">
+        <v>180</v>
       </c>
       <c r="S13" t="n">
-        <v>150</v>
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>92.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Lucero Martínez</t>
+        </is>
+      </c>
       <c r="X13" t="n">
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Felipe Hernández</t>
+        </is>
+      </c>
       <c r="AB13" t="n">
         <v>0</v>
       </c>
       <c r="AC13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Fernando García</t>
+        </is>
+      </c>
       <c r="AF13" t="n">
         <v>0</v>
       </c>
       <c r="AG13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Control de Calidad</t>
+        </is>
+      </c>
       <c r="AJ13" t="n">
         <v>0</v>
       </c>
       <c r="AK13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>Acabados Finales</t>
+        </is>
+      </c>
       <c r="AN13" t="n">
         <v>0</v>
       </c>
       <c r="AO13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
@@ -1951,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: resolved issues and polished UI interactions
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -709,17 +709,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>fewygfyu3</t>
+          <t>JCI240001A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HVAC-CTL-TEST-001</t>
+          <t>HVAC-CTL-2024-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Controlador HVAC Premium</t>
+          <t>Controlador HVAC Inteligente</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -729,205 +729,185 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>WO-TEST-0001</t>
+          <t>WO-2024-0156</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BTH-TEST001</t>
+          <t>BTH-240001</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SNTEST001</t>
+          <t>SN240001001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TEST-MX</t>
+          <t>FORD-MX</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Rev-A</t>
+          <t>Rev-C</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>JCI-SPEC-HVAC-TEST-A</t>
+          <t>JCI-SPEC-HVAC-2024-A</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>45903.96087520188</v>
+        <v>45905.02126497685</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>45905.02247832176</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>45905.02336631944</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>45903.96087520188</v>
+        <v>45905.02336631944</v>
       </c>
       <c r="R2" t="n">
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U2" t="n">
-        <v>100</v>
+        <v>93.23380730617255</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X2" t="n">
         <v>0</v>
       </c>
       <c r="Y2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF2" t="n">
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ2" t="n">
         <v>0</v>
       </c>
       <c r="AK2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
       <c r="AO2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="n">
         <v>0</v>
       </c>
       <c r="AS2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JCI240001A</t>
+          <t>JCI240002B</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HVAC-CTL-2024-001</t>
+          <t>BATT-SYS-2024-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Controlador HVAC Inteligente</t>
+          <t>Sistema de Gestión de Batería</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Controles HVAC</t>
+          <t>Sistemas de Energía</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>WO-2024-0156</t>
+          <t>WO-2024-0157</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>BTH-240001</t>
+          <t>BTH-240002</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SN240001001</t>
+          <t>SN240002001</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FORD-MX</t>
+          <t>GM-MX</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Rev-C</t>
+          <t>Rev-B</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>JCI-SPEC-HVAC-2024-A</t>
+          <t>JCI-SPEC-BATT-2024-B</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -939,16 +919,19 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>45903.96087520155</v>
+        <v>45905.02126516363</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>45905.02249077546</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>45903.96087520156</v>
+        <v>45905.02249078052</v>
       </c>
       <c r="R3" t="n">
-        <v>420</v>
+        <v>380</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -957,87 +940,67 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>100</v>
+        <v>93.46909736051569</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
         <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
+      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="n">
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
+      <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="n">
         <v>0</v>
       </c>
       <c r="AK3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
+      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="n">
         <v>0</v>
       </c>
       <c r="AO3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -1049,79 +1012,82 @@
         <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JCI240002B</t>
+          <t>fewygfyu3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BATT-SYS-2024-002</t>
+          <t>HVAC-CTL-TEST-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sistema de Gestión de Batería</t>
+          <t>Controlador HVAC Premium</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sistemas de Energía</t>
+          <t>Controles HVAC</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>WO-2024-0157</t>
+          <t>WO-TEST-0001</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BTH-240002</t>
+          <t>BTH-TEST001</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>SN240002001</t>
+          <t>SNTEST001</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>GM-MX</t>
+          <t>TEST-MX</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Rev-B</t>
+          <t>Rev-A</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>JCI-SPEC-BATT-2024-B</t>
+          <t>JCI-SPEC-HVAC-TEST-A</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>45903.96087520177</v>
+        <v>45905.02126516204</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>45905.02250319444</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>45903.96087520178</v>
+        <v>45905.02250319444</v>
       </c>
       <c r="R4" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -1130,99 +1096,73 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>100</v>
+        <v>96.75748304699992</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB4" t="n">
         <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF4" t="n">
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
       <c r="AK4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="n">
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1285,13 +1225,13 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>45903.960875202</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>45903.960875202</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R5" t="n">
         <v>280</v>
@@ -1310,92 +1250,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB5" t="n">
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF5" t="n">
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ5" t="n">
         <v>0</v>
       </c>
       <c r="AK5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN5" t="n">
         <v>0</v>
       </c>
       <c r="AO5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="n">
         <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1458,13 +1372,13 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>45903.96087520209</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>45903.96087520209</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R6" t="n">
         <v>250</v>
@@ -1483,92 +1397,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB6" t="n">
         <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF6" t="n">
         <v>0</v>
       </c>
       <c r="AG6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ6" t="n">
         <v>0</v>
       </c>
       <c r="AK6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN6" t="n">
         <v>0</v>
       </c>
       <c r="AO6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="n">
         <v>0</v>
       </c>
       <c r="AS6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1631,13 +1519,13 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>45903.96087520219</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>45903.9608752022</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R7" t="n">
         <v>300</v>
@@ -1656,92 +1544,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB7" t="n">
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF7" t="n">
         <v>0</v>
       </c>
       <c r="AG7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
       <c r="AK7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN7" t="n">
         <v>0</v>
       </c>
       <c r="AO7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="n">
         <v>0</v>
       </c>
       <c r="AS7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1804,13 +1666,13 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>45903.96087520227</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>45903.96087520227</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R8" t="n">
         <v>350</v>
@@ -1829,92 +1691,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X8" t="n">
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB8" t="n">
         <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ8" t="n">
         <v>0</v>
       </c>
       <c r="AK8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN8" t="n">
         <v>0</v>
       </c>
       <c r="AO8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="n">
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1977,13 +1813,13 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>45903.96087520237</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>45903.96087520239</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R9" t="n">
         <v>220</v>
@@ -2002,92 +1838,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB9" t="n">
         <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF9" t="n">
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ9" t="n">
         <v>0</v>
       </c>
       <c r="AK9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN9" t="n">
         <v>0</v>
       </c>
       <c r="AO9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="n">
         <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2150,13 +1960,13 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>45903.96087520247</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>45903.96087520247</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R10" t="n">
         <v>290</v>
@@ -2175,92 +1985,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X10" t="n">
         <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB10" t="n">
         <v>0</v>
       </c>
       <c r="AC10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF10" t="n">
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
       <c r="AK10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN10" t="n">
         <v>0</v>
       </c>
       <c r="AO10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="n">
         <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2323,13 +2107,13 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>45903.96087520256</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>45903.96087520257</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R11" t="n">
         <v>410</v>
@@ -2348,92 +2132,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB11" t="n">
         <v>0</v>
       </c>
       <c r="AC11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF11" t="n">
         <v>0</v>
       </c>
       <c r="AG11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ11" t="n">
         <v>0</v>
       </c>
       <c r="AK11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN11" t="n">
         <v>0</v>
       </c>
       <c r="AO11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="n">
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2496,13 +2254,13 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>45903.96087520264</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>45903.96087520264</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="R12" t="n">
         <v>365</v>
@@ -2521,92 +2279,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X12" t="n">
         <v>0</v>
       </c>
       <c r="Y12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI12" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ12" t="n">
         <v>0</v>
       </c>
       <c r="AK12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN12" t="n">
         <v>0</v>
       </c>
       <c r="AO12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="n">
         <v>0</v>
       </c>
       <c r="AS12" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2669,13 +2401,13 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>45903.96087520272</v>
+        <v>45905.02126517361</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>45903.96087520272</v>
+        <v>45905.02126517361</v>
       </c>
       <c r="R13" t="n">
         <v>180</v>
@@ -2694,92 +2426,66 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>Lucero Martínez</t>
-        </is>
-      </c>
       <c r="X13" t="n">
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>Felipe Hernández</t>
-        </is>
-      </c>
       <c r="AB13" t="n">
         <v>0</v>
       </c>
       <c r="AC13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>Fernando García</t>
-        </is>
-      </c>
       <c r="AF13" t="n">
         <v>0</v>
       </c>
       <c r="AG13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>Control de Calidad</t>
-        </is>
-      </c>
       <c r="AJ13" t="n">
         <v>0</v>
       </c>
       <c r="AK13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>Acabados Finales</t>
-        </is>
-      </c>
       <c r="AN13" t="n">
         <v>0</v>
       </c>
       <c r="AO13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="n">
         <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stable: dynamic system reaching a more stable version
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -766,31 +766,31 @@
         <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>45905.02126497685</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>45905.02247832176</v>
+        <v>45905.30400947916</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>45905.02336631944</v>
+        <v>45905.30967788195</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>45905.02336631944</v>
+        <v>45905.30967788195</v>
       </c>
       <c r="R2" t="n">
         <v>420</v>
       </c>
       <c r="S2" t="n">
-        <v>76</v>
+        <v>489</v>
       </c>
       <c r="T2" t="n">
-        <v>100</v>
+        <v>85.88957055214725</v>
       </c>
       <c r="U2" t="n">
-        <v>93.23380730617255</v>
+        <v>94.65752305073333</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -912,23 +912,23 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="M3" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>45905.02126516363</v>
+        <v>45905.02126516204</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>45905.02249077546</v>
+        <v>45905.30485422454</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>45905.02249078052</v>
+        <v>45905.3100958912</v>
       </c>
       <c r="R3" t="n">
         <v>380</v>
@@ -940,14 +940,13 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>93.46909736051569</v>
+        <v>92.00444548937793</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
         <v>0</v>
       </c>
@@ -959,7 +958,6 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
@@ -971,7 +969,6 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="n">
         <v>0</v>
       </c>
@@ -983,7 +980,6 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="n">
         <v>0</v>
       </c>
@@ -995,7 +991,6 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="n">
         <v>0</v>
       </c>
@@ -1007,7 +1002,6 @@
           <t>No Iniciado</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="n">
         <v>0</v>
       </c>
@@ -1365,20 +1359,23 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>45905.02126516204</v>
       </c>
+      <c r="O6" s="2" t="n">
+        <v>45905.27189943287</v>
+      </c>
       <c r="Q6" s="2" t="n">
-        <v>45905.02126516204</v>
+        <v>45905.27189943287</v>
       </c>
       <c r="R6" t="n">
         <v>250</v>
@@ -1390,7 +1387,7 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>100</v>
+        <v>92.77052788714585</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1512,20 +1509,23 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="M7" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>45905.02126516204</v>
+        <v>45905.02126516494</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>45905.31726680831</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>45905.02126516204</v>
+        <v>45905.3175695747</v>
       </c>
       <c r="R7" t="n">
         <v>300</v>
@@ -1537,13 +1537,14 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>100</v>
+        <v>91.7062103974647</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="n">
         <v>0</v>
       </c>
@@ -1555,6 +1556,7 @@
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="n">
         <v>0</v>
       </c>
@@ -1566,6 +1568,7 @@
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="n">
         <v>0</v>
       </c>
@@ -1577,6 +1580,7 @@
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
@@ -1588,6 +1592,7 @@
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="n">
         <v>0</v>
       </c>
@@ -1599,6 +1604,7 @@
           <t>No Iniciado</t>
         </is>
       </c>
+      <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="n">
         <v>0</v>
       </c>
@@ -1659,20 +1665,23 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="M8" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>45905.02126516204</v>
       </c>
+      <c r="O8" s="2" t="n">
+        <v>45905.29023958333</v>
+      </c>
       <c r="Q8" s="2" t="n">
-        <v>45905.02126516204</v>
+        <v>45905.29159174769</v>
       </c>
       <c r="R8" t="n">
         <v>350</v>
@@ -1684,7 +1693,7 @@
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>100</v>
+        <v>93.09553997225412</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
stable: correction reset products
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS13"/>
+  <dimension ref="A1:AS14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="45"/>
@@ -718,20 +718,23 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>45903.96087520188</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>45908.42248816912</v>
+      </c>
       <c r="Q2" s="3" t="n">
-        <v>45903.96087520188</v>
+        <v>45908.42248816953</v>
       </c>
       <c r="R2" t="n">
         <v>300</v>
@@ -743,7 +746,7 @@
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>100</v>
+        <v>96.86870964452501</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -878,7 +881,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="N3" s="3" t="n">
         <v>45903.96087520155</v>
@@ -1031,7 +1034,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>45903.96087520177</v>
@@ -1184,7 +1187,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>45903.960875202</v>
@@ -1337,7 +1340,7 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>45903.96087520209</v>
@@ -1490,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>45903.96087520219</v>
@@ -1643,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>45903.96087520227</v>
@@ -1796,7 +1799,7 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N9" s="3" t="n">
         <v>45903.96087520237</v>
@@ -1949,7 +1952,7 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>45903.96087520247</v>
@@ -2102,7 +2105,7 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>45903.96087520256</v>
@@ -2255,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N12" s="3" t="n">
         <v>45903.96087520264</v>
@@ -2408,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N13" s="3" t="n">
         <v>45903.96087520272</v>
@@ -2498,6 +2501,159 @@
         <v>0</v>
       </c>
       <c r="AS13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TEST12345</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PN-001</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Producto Test</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Familia Test</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>WO-001</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SN001</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Rev1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Spec A</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>45908.41174113636</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>45908.41201844931</v>
+      </c>
+      <c r="R14" t="n">
+        <v>300</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>100</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>No Iniciado</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
release: prepared stable build of system ready for demo presentation
</commit_message>
<xml_diff>
--- a/data/excel/DATOS_JCI_PROYECTO.xlsx
+++ b/data/excel/DATOS_JCI_PROYECTO.xlsx
@@ -718,35 +718,38 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>16.66666666666666</v>
+        <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>45903.96087520188</v>
+        <v>45908.52342356316</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>45908.42248816912</v>
+        <v>45908.52383052128</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>45908.52461455095</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>45908.42248816953</v>
+        <v>45908.52461455098</v>
       </c>
       <c r="R2" t="n">
         <v>300</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U2" t="n">
-        <v>96.86870964452501</v>
+        <v>93.1021239710109</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -884,10 +887,10 @@
         <v>20</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>45903.96087520155</v>
+        <v>45908.52342356156</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>45903.96087520156</v>
+        <v>45908.52342356157</v>
       </c>
       <c r="R3" t="n">
         <v>420</v>
@@ -1037,10 +1040,10 @@
         <v>20</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>45903.96087520177</v>
+        <v>45908.52342356263</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>45903.96087520178</v>
+        <v>45908.52342356264</v>
       </c>
       <c r="R4" t="n">
         <v>380</v>
@@ -1180,32 +1183,38 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>45903.960875202</v>
+        <v>45908.52342356376</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>45908.52394916852</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>45908.52512879029</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>45903.960875202</v>
+        <v>45908.52512879032</v>
       </c>
       <c r="R5" t="n">
         <v>280</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U5" t="n">
-        <v>100</v>
+        <v>93.971020483174</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -1343,10 +1352,10 @@
         <v>20</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>45903.96087520209</v>
+        <v>45908.52342356431</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>45903.96087520209</v>
+        <v>45908.52342356434</v>
       </c>
       <c r="R6" t="n">
         <v>250</v>
@@ -1496,10 +1505,10 @@
         <v>20</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>45903.96087520219</v>
+        <v>45908.52342356509</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>45903.9608752022</v>
+        <v>45908.52342356509</v>
       </c>
       <c r="R7" t="n">
         <v>300</v>
@@ -1649,10 +1658,10 @@
         <v>20</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>45903.96087520227</v>
+        <v>45908.52342356558</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>45903.96087520227</v>
+        <v>45908.52342356559</v>
       </c>
       <c r="R8" t="n">
         <v>350</v>
@@ -1802,10 +1811,10 @@
         <v>20</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>45903.96087520237</v>
+        <v>45908.52342356605</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>45903.96087520239</v>
+        <v>45908.52342356607</v>
       </c>
       <c r="R9" t="n">
         <v>220</v>
@@ -1955,10 +1964,10 @@
         <v>20</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>45903.96087520247</v>
+        <v>45908.52342356658</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>45903.96087520247</v>
+        <v>45908.52342356658</v>
       </c>
       <c r="R10" t="n">
         <v>290</v>
@@ -2108,10 +2117,10 @@
         <v>20</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>45903.96087520256</v>
+        <v>45908.52342356719</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>45903.96087520257</v>
+        <v>45908.52342356719</v>
       </c>
       <c r="R11" t="n">
         <v>410</v>
@@ -2261,10 +2270,10 @@
         <v>20</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>45903.96087520264</v>
+        <v>45908.52342356768</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>45903.96087520264</v>
+        <v>45908.52342356768</v>
       </c>
       <c r="R12" t="n">
         <v>365</v>
@@ -2414,10 +2423,10 @@
         <v>20</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>45903.96087520272</v>
+        <v>45908.52342356815</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>45903.96087520272</v>
+        <v>45908.52342356815</v>
       </c>
       <c r="R13" t="n">
         <v>180</v>

</xml_diff>